<commit_message>
features : mercahnt info logic
</commit_message>
<xml_diff>
--- a/reports/excel/698167220.xlsx
+++ b/reports/excel/698167220.xlsx
@@ -549,21 +549,22 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The customer's income and credit profile indicate an average monthly cash flow of ₹50,922, with an average net inflow of ₹313,622 and outflow of ₹8,090. Their salary income is ₹51,020 on average from six transactions, while their EMI commitments amount to ₹7,500 per payment, with two debit transactions occurring each month. The customer's key spending categories include other expenses at ₹8,045 and mobility costs at ₹45.
-The customer's tradeline portfolio consists of N=27 total tradelines, M=22 live tradelines, and P=5 closed tradelines. The portfolio features a mix of credit card (26 accounts) and personal loan (1 account) products, with sanctioned exposure totaling INR 72,48,130 and outstanding balances of INR 8,22,679 for the entire portfolio, and INR 3,11,925 for the personal loan product. The customer's credit utilization percentage is 9.0% for credit cards, indicating a relatively healthy balance. The customer has a low-risk profile, with no missed payments, minimal enquiry pressure, and stable loan acquisition velocity.</t>
+          <t>The customer's income is ₹51,020 per month, sourced from six transactions, resulting in an average net cash flow of ₹50,922. Their key spending categories include other expenses at ₹8,045 and mobility costs at ₹45. The customer has EMI commitments averaging ₹7,500 per payment, with two debit transactions per month.
+The customer's tradeline portfolio consists of N=27 total tradelines (M live=22, P closed=5). The portfolio features a mix of loan products, with Credit Card being the dominant product type, accounting for 26 live accounts. Total sanctioned exposure stands at INR 72,48,130, while total outstanding is INR 8,22,679. Unsecured sanction amount and outstanding are identical to total outstanding, indicating no separation between secured and unsecured loans. The credit card utilization percentage is 9.0%, which is elevated. The customer's creditworthiness assessment is cautious.
+Note: This is a synthesised summary based on automated banking and bureau analyses. Independent verification is recommended before final credit decisions.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Here is the executive summary:
-The customer's tradeline portfolio consists of N=27 total tradelines, M=22 live tradelines, and P=5 closed tradelines. The portfolio features a mix of credit card (26 accounts) and personal loan (1 account) products, with sanctioned exposure totaling INR 72,48,130 and outstanding balances of INR 8,22,679 for the entire portfolio, and INR 3,11,925 for the personal loan product. The customer's credit utilization percentage is 9.0% for credit cards, indicating a relatively healthy balance. Notably, there are no DPD values above zero, suggesting a clean payment history.
-The customer's behavioral features indicate a low-risk profile. The % Missed Payments Last 18M is 0.00%, indicating no missed payments, and the Trade-to-Enquiry Ratio (Unsec 24M) is 40.00%, which is within healthy limits. The CC Balance Utilization is 8.97%, and the PL Balance Remaining is 53.46%, with the latter being moderate but not concerning. The customer has a low enquiry activity, with Unsecured Enquiries Last 12M at 0, indicating minimal enquiry pressure. The Avg Interpurchase Time All Loans (24M) is 3.45 months, suggesting a relatively stable loan acquisition velocity. Overall, the customer's credit behavior suggests a low-risk profile.</t>
+The customer's tradeline portfolio consists of N=27 total tradelines (M live=22, P closed=5). The portfolio features a mix of loan products, with Credit Card being the dominant product type, accounting for 26 live accounts. Total sanctioned exposure stands at INR 72,48,130, while total outstanding is INR 8,22,679. Unsecured sanction amount and outstanding are identical to total outstanding, indicating no separation between secured and unsecured loans. The credit card utilization percentage is 9.0%, which is elevated. There are no defaulted loan types present in the data.
+The customer's behavioral features indicate a relatively clean repayment profile, with zero DPD across all products and windows, no missed payments. The trade-to-enquiry ratio is 40.00% for unsecured trades, indicating moderate enquiry activity. Loan acquisition velocity is also notable, with an average interpurchase time of 3.45 months. However, the sanctioned exposure trend shows a decrease in sanctioned exposure over the past 12 and 6 months, from ₹66.6L to ₹64.1L and ₹66.6L to ₹64.3L respectively, indicating some stability in the trend.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>The customer's banking profile indicates a monthly cash flow of ₹50,922, with an average net inflow of ₹313,622 and outflow of ₹8,090. Their salary income is ₹51,020 on average from six transactions, while their EMI commitments amount to ₹7,500 per payment, with two debit transactions occurring each month. The customer's key spending categories include other expenses at ₹8,045 and mobility costs at ₹45.
-The customer received a salary of ₹72,000 in Jun 2025 and transferred ₹72,000 to their own account the next day. In Jul 2025, the customer made four transactions with BHOSALE RAJU TA, totaling ₹800. In Aug 2025, the customer received ₹51,020 from their salary income and paid ₹7,500 in EMI.</t>
+          <t>The customer's banking profile presents a stable financial picture. Their average monthly salary is ₹51,020, sourced from six transactions, resulting in an average net cash flow of ₹50,922. This translates to a total inflow of ₹313,622 and an outflow of ₹8,090 per month. The customer's key spending categories include other expenses at ₹8,045 and mobility costs at ₹45. Additionally, the customer has EMI commitments averaging ₹7,500 per payment, with two debit transactions per month.
+The customer's banking profile also reveals some notable merchant activity. The most frequent merchant is BHOSALE RAJU TA, with four transactions totaling ₹800. Furthermore, the account appears to be their primary account, as EMI payments are visible and average two debit transactions per month. Notably, the customer has a Banking FOIR obligation-to-income ratio of 14.7%, which falls within the comfortable range.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">

</xml_diff>

<commit_message>
added the log of deepseek think
</commit_message>
<xml_diff>
--- a/reports/excel/698167220.xlsx
+++ b/reports/excel/698167220.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
prompt, sort filter in checklist, reasoning log
</commit_message>
<xml_diff>
--- a/reports/excel/698167220.xlsx
+++ b/reports/excel/698167220.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>